<commit_message>
feat: initialize OBE 2026 curriculum documentation, including structural analysis, assessment frameworks, and competency mappings
</commit_message>
<xml_diff>
--- a/KURIKULUM2026_REVISI/005_STRUKTUR_KURIKULUM_8_SEMESTER_DAN_PEMINATAN.xlsx
+++ b/KURIKULUM2026_REVISI/005_STRUKTUR_KURIKULUM_8_SEMESTER_DAN_PEMINATAN.xlsx
@@ -1865,7 +1865,7 @@
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>SEMESTER 3 (20 SKS) — Penguatan Core RPL, OS &amp; Jaringan Komputer</t>
+          <t>SEMESTER 3 (20 SKS) — Penguatan Core RPL, OS, Jarkom &amp; UI/UX</t>
         </is>
       </c>
       <c r="B52" s="4" t="n"/>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="G54" s="7" t="inlineStr">
         <is>
-          <t>`STI-104`, `FST-207`</t>
+          <t>`STI-101`, `FST-207`</t>
         </is>
       </c>
     </row>
@@ -1962,17 +1962,17 @@
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>Kecerdasan Buatan (Artificial Intelligence)</t>
+          <t>Sistem Cerdas</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>+P</t>
+          <t>Teori</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr">
@@ -1982,7 +1982,7 @@
       </c>
       <c r="G55" s="9" t="inlineStr">
         <is>
-          <t>`STI-201`, `STI-202`</t>
+          <t>`STI-201`, `FST-204`</t>
         </is>
       </c>
     </row>
@@ -1999,7 +1999,7 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>Desain Pengalaman Pengguna (UI/UX Design)</t>
+          <t>UI/UX Design &amp; Prototyping</t>
         </is>
       </c>
       <c r="D56" s="8" t="inlineStr">
@@ -2019,7 +2019,7 @@
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>`STI-104`</t>
+          <t>`FST-101`</t>
         </is>
       </c>
     </row>
@@ -2056,7 +2056,7 @@
       </c>
       <c r="G57" s="9" t="inlineStr">
         <is>
-          <t>`STI-202`</t>
+          <t>`FST-203`</t>
         </is>
       </c>
     </row>
@@ -2093,7 +2093,7 @@
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>`STI-201`</t>
+          <t>`STI-103`</t>
         </is>
       </c>
     </row>
@@ -2110,12 +2110,12 @@
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>Pemrograman Web Front-End</t>
+          <t>Web Front End Development</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
-          <t>`STI-202`</t>
+          <t>`FST-102`</t>
         </is>
       </c>
     </row>
@@ -2167,7 +2167,7 @@
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>`STI-104`</t>
+          <t>`STI-103`</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: align Dok 005 with all markdown files, fix STI-625 SKS and cumulative arithmetic
</commit_message>
<xml_diff>
--- a/KURIKULUM2026_REVISI/005_STRUKTUR_KURIKULUM_8_SEMESTER_DAN_PEMINATAN.xlsx
+++ b/KURIKULUM2026_REVISI/005_STRUKTUR_KURIKULUM_8_SEMESTER_DAN_PEMINATAN.xlsx
@@ -558,8 +558,8 @@
     <col width="56.34999999999999" customWidth="1" min="2" max="2"/>
     <col width="69" customWidth="1" min="3" max="3"/>
     <col width="40.25" customWidth="1" min="4" max="4"/>
-    <col width="50.59999999999999" customWidth="1" min="5" max="5"/>
-    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="69" customWidth="1" min="5" max="5"/>
+    <col width="54.05" customWidth="1" min="6" max="6"/>
     <col width="35.65" customWidth="1" min="7" max="7"/>
     <col width="47.15" customWidth="1" min="8" max="8"/>
   </cols>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>Deep Learning &amp; IoT</t>
+          <t>Keamanan Lanjut &amp; IoT</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
@@ -3110,7 +3110,7 @@
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>Deep Learning, IoT, Mobile, KPM, Peminatan 1</t>
+          <t>Keamanan Lanjut, Data Mining, IoT, Mobile, KPM, Peminatan 1</t>
         </is>
       </c>
     </row>
@@ -3122,7 +3122,7 @@
       </c>
       <c r="B84" s="9" t="inlineStr">
         <is>
-          <t>AI Integrasi &amp; Platform</t>
+          <t>Deep Learning &amp; Platform</t>
         </is>
       </c>
       <c r="C84" s="10" t="inlineStr">
@@ -3137,7 +3137,7 @@
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>Smart AI, Smart City, Platform, Metopel</t>
+          <t>Integrasi AI, Smart City, Deep Learning, Platform Eng, Metopen</t>
         </is>
       </c>
     </row>
@@ -4762,7 +4762,7 @@
     <row r="137" ht="20" customHeight="1">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>SEMESTER 5 (21 SKS) — Tahap Spesialisasi Deep Learning, IoT &amp; Peminatan 1</t>
+          <t>SEMESTER 5 (21 SKS) — Tahap Spesialisasi Keamanan Lanjut, IoT &amp; Peminatan 1</t>
         </is>
       </c>
       <c r="B137" s="4" t="n"/>
@@ -5146,7 +5146,7 @@
     <row r="149" ht="20" customHeight="1">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>SEMESTER 6 (19 SKS) — Tahap Spesialisasi MBKM &amp; Platform Engineering</t>
+          <t>SEMESTER 6 (19 SKS) — Tahap Spesialisasi Deep Learning, Platform Engineering &amp; MBKM</t>
         </is>
       </c>
       <c r="B149" s="4" t="n"/>
@@ -6162,7 +6162,7 @@
       </c>
       <c r="F182" s="7" t="inlineStr">
         <is>
-          <t>Tahap Spesialisasi Deep Learning &amp; IoT</t>
+          <t>Tahap Spesialisasi Keamanan Lanjut &amp; IoT</t>
         </is>
       </c>
     </row>
@@ -6194,7 +6194,7 @@
       </c>
       <c r="F183" s="9" t="inlineStr">
         <is>
-          <t>Tahap Spesialisasi MBKM &amp; Platform Eng</t>
+          <t>Tahap Spesialisasi Deep Learning &amp; Platform Eng</t>
         </is>
       </c>
     </row>

</xml_diff>